<commit_message>
Agregar descarga de todos los QR en un solo ZIP desde el panel
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/prueba_100_productos.xlsx
+++ b/data/prueba_100_productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valentinatorres/Downloads/BestPrice-QR/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66CA8344-FBB5-2A49-9AE3-50AAFB3F7A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DCF184-716D-AB41-8132-56A27F822E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="340" yWindow="1900" windowWidth="17160" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="291">
   <si>
     <t>SKU</t>
   </si>
@@ -890,6 +890,9 @@
   </si>
   <si>
     <t>Oreo</t>
+  </si>
+  <si>
+    <t>Imagen URL</t>
   </si>
 </sst>
 </file>
@@ -1245,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1262,7 +1265,7 @@
     <col min="12" max="12" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1299,8 +1302,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M1" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1326,7 +1332,7 @@
         <v>13.22</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1352,7 +1358,7 @@
         <v>7.56</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1384,7 +1390,7 @@
         <v>4.6399999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1422,7 +1428,7 @@
         <v>3.97</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1454,7 +1460,7 @@
         <v>15.74</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1486,7 +1492,7 @@
         <v>9.81</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1518,7 +1524,7 @@
         <v>6.19</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1550,7 +1556,7 @@
         <v>12.85</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1582,7 +1588,7 @@
         <v>29.56</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1608,7 +1614,7 @@
         <v>23.77</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1646,7 +1652,7 @@
         <v>4.2699999999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1678,7 +1684,7 @@
         <v>5.22</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -1710,7 +1716,7 @@
         <v>13.25</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -1742,7 +1748,7 @@
         <v>12.27</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>56</v>
       </c>

</xml_diff>